<commit_message>
Correct design hold to 1–3 months and add rainfall-to-fill method
The Afghan check dams are rainfall-fed and meant to stay full about
one to three months, not a few hours. Document the parameters that
control storage duration, add SCS-CN rainfall to fill 100%, and put
both in the workbook FillAndHold sheet. Daily Form B is the default
pond log; Annex A is only for gabion/leaky outliers.

Co-authored-by: Maziarkarimi88 <Maziarkarimi88@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/CheckDam_Recharge_Calculator.xlsx
+++ b/templates/CheckDam_Recharge_Calculator.xlsx
@@ -15,8 +15,9 @@
     <sheet name="DailyCalc" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Wells" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Karez" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Summary" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Scorecard" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="FillAndHold" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Summary" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Scorecard" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="MeanMDWIR">DailyCalc!$S$1</definedName>
@@ -849,7 +850,7 @@
     <row r="2" ht="48" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Field workbook for small check dams on Kandahar / Zabul alluvial fans. Yellow cells are inputs. Blue cells are formulas — do not type over them. An example spring filling is pre-loaded so you can see a complete result; replace it with your Form B and Form C data.</t>
+          <t>Field workbook for rainfall-fed check dams designed to hold about 1–3 months when full. Yellow cells are inputs. Blue cells are formulas — do not type over them. An example spring filling is pre-loaded so you can see a complete result; replace it with your Form B and Form C data. Sheet FillAndHold estimates rainfall to fill 100%.</t>
         </is>
       </c>
     </row>
@@ -882,7 +883,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Names, crest, Sy, default evaporation. Matches Form A.</t>
+          <t>Names, crest, catchment ha, Sy. Matches Form A.</t>
         </is>
       </c>
     </row>
@@ -901,82 +902,94 @@
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
         <is>
-          <t>3. Evaporation</t>
+          <t>3. FillAndHold</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Monthly open-water E (mm/day). Override if you have a pan (use 0.7 × pan).</t>
+          <t>Rainfall (mm) to fill 100%; days to empty from full (1–3 month check).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>4. DailyPond</t>
+          <t>4. Evaporation</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
         <is>
-          <t>Paste Form B: date, rain, stage, overflow, pumped.</t>
+          <t>Monthly open-water E (mm/day). Override if you have a pan (use 0.7 × pan).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>5. DailyCalc</t>
+          <t>5. DailyPond</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>Interpolates A and V, flags dry days, computes MDWIR and daily infiltration.</t>
+          <t>Paste Form B: date, rain, stage, overflow, pumped.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>6. Wells</t>
+          <t>6. DailyCalc</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Form C water levels. Converts DTW to elevation and seasonal Δh.</t>
+          <t>Interpolates A and V, flags dry days, computes MDWIR and daily infiltration.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>7. Karez</t>
+          <t>7. Wells</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Weekly KO discharge and flow-day count.</t>
+          <t>Form C water levels. Converts DTW to elevation and seasonal Δh.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>8. Summary</t>
+          <t>8. Karez</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>I1–I5 for the year.</t>
+          <t>Weekly KO discharge and flow-day count.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>9. Scorecard</t>
+          <t>9. Summary</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t>I1–I5 for the year.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>10. Scorecard</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>Interpretation and desilting decision.</t>
         </is>
@@ -1058,6 +1071,517 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="001D5673"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="62" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Annual summary — I1 to I5</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3">
+        <f>CONCATENATE("Dam ",Site!B4," — ",Site!B5," — ",Site!B6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Indicator</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Unit</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>How it is computed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="33" t="inlineStr">
+        <is>
+          <t>I1</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>Infiltration volume</t>
+        </is>
+      </c>
+      <c r="C5" s="18">
+        <f>DailyCalc!S2</f>
+        <v/>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Sum of daily infiltration (dry-day storage drop − E, else MDWIR × A)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="33" t="inlineStr">
+        <is>
+          <t>I2</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>Fillings per year</t>
+        </is>
+      </c>
+      <c r="C6" s="25">
+        <f>IF(StageAreaVolume!B20=0,"",C5/StageAreaVolume!B20)</f>
+        <v/>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>I1 / crest storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="33" t="inlineStr">
+        <is>
+          <t>I3</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>Mean MDWIR</t>
+        </is>
+      </c>
+      <c r="C7" s="18">
+        <f>DailyCalc!S1</f>
+        <v/>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>mm/day</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Average dry-day infiltration rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="34" t="inlineStr"/>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Mean E while ponded</t>
+        </is>
+      </c>
+      <c r="C8" s="18">
+        <f>IFERROR(AVERAGEIF(DailyCalc!C5:C204,"&gt;0",DailyCalc!G5:G204),0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="5" t="inlineStr">
+        <is>
+          <t>mm/day</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>Evaporation on days with water</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="34" t="inlineStr"/>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>MDWIR / E</t>
+        </is>
+      </c>
+      <c r="C9" s="25">
+        <f>IF(C8=0,"",C7/C8)</f>
+        <v/>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Healthy gravel beds are often 4–8</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="33" t="inlineStr">
+        <is>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>Extra water-table rise vs control</t>
+        </is>
+      </c>
+      <c r="C10" s="25">
+        <f>Wells!L17</f>
+        <v/>
+      </c>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>Mean Δh of W-N and W-M minus mean Δh of C</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="34" t="inlineStr"/>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>Recharge depth (Sy default)</t>
+        </is>
+      </c>
+      <c r="C11" s="18">
+        <f>Wells!L18</f>
+        <v/>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>Sy × I4; not a volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="34" t="inlineStr"/>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>Recharge depth range</t>
+        </is>
+      </c>
+      <c r="C12" s="35">
+        <f>TEXT(Wells!L19,"0.0")&amp;" – "&amp;TEXT(Wells!L20,"0.0")</f>
+        <v/>
+      </c>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>Sy low to Sy high</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="33" t="inlineStr">
+        <is>
+          <t>I5</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>Extra karez flow-day visits</t>
+        </is>
+      </c>
+      <c r="C13" s="25">
+        <f>Karez!I7</f>
+        <v/>
+      </c>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>visits</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>Treated flowing visits − control flowing visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="34" t="inlineStr"/>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>Extra karez days if weekly</t>
+        </is>
+      </c>
+      <c r="C14" s="25">
+        <f>C13*7</f>
+        <v/>
+      </c>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>Assumes weekly KO visits</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="34" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Mean KO discharge while flowing</t>
+        </is>
+      </c>
+      <c r="C15" s="25">
+        <f>Karez!I5</f>
+        <v/>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>L/s</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
+        <is>
+          <t>Average of Q &gt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="34" t="inlineStr"/>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>Days with water in pond</t>
+        </is>
+      </c>
+      <c r="C16" s="25">
+        <f>DailyCalc!S3</f>
+        <v/>
+      </c>
+      <c r="D16" s="5" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
+        <is>
+          <t>Stage &gt; 0</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="34" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Dry days used for MDWIR</t>
+        </is>
+      </c>
+      <c r="C17" s="25">
+        <f>DailyCalc!S4</f>
+        <v/>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>days</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Should be as many as possible</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="34" t="inlineStr"/>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>Crest storage</t>
+        </is>
+      </c>
+      <c r="C18" s="18">
+        <f>StageAreaVolume!B20</f>
+        <v/>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E18" s="6" t="inlineStr">
+        <is>
+          <t>From survey</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="34" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Catchment rain in DailyPond</t>
+        </is>
+      </c>
+      <c r="C19" s="18">
+        <f>SUM(DailyPond!B5:B204)</f>
+        <v/>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>Village gauge total for logged days</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="34" t="inlineStr"/>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>I1 as depth on catchment</t>
+        </is>
+      </c>
+      <c r="C20" s="18">
+        <f>IF(Site!B14=0,"",C5/(Site!B14*10))</f>
+        <v/>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>mm</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>m³ / (ha × 10) = mm</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Workbook vs independent Python check (example dataset only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Python I1 (m³)</t>
+        </is>
+      </c>
+      <c r="B24" s="18" t="n">
+        <v>6365.418698335041</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Workbook I1 − Python</t>
+        </is>
+      </c>
+      <c r="D24" s="18">
+        <f>C5-B24</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Python mean MDWIR (mm/d)</t>
+        </is>
+      </c>
+      <c r="B25" s="25" t="n">
+        <v>48.21522767955886</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Workbook MDWIR − Python</t>
+        </is>
+      </c>
+      <c r="D25" s="25">
+        <f>C7-B25</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Python I4 (m)</t>
+        </is>
+      </c>
+      <c r="B26" s="36" t="n">
+        <v>1.025</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Workbook I4 − Python</t>
+        </is>
+      </c>
+      <c r="D26" s="36">
+        <f>C10-B26</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>If the example is still loaded, differences should be near zero (interpolation rounding &lt; ~2%). After you replace the example, ignore this block.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A27:E28"/>
+    <mergeCell ref="A2:D2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00B0894A"/>
@@ -23617,508 +24141,314 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="001D5673"/>
+    <tabColor rgb="002A9D8F"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Annual summary — I1 to I5</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3">
-        <f>CONCATENATE("Dam ",Site!B4," — ",Site!B5," — ",Site!B6)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4" ht="28" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>ID</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>Indicator</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>Unit</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>How it is computed</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="33" t="inlineStr">
-        <is>
-          <t>I1</t>
-        </is>
-      </c>
-      <c r="B5" s="5" t="inlineStr">
-        <is>
-          <t>Infiltration volume</t>
-        </is>
-      </c>
-      <c r="C5" s="18">
-        <f>DailyCalc!S2</f>
-        <v/>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>Sum of daily infiltration (dry-day storage drop − E, else MDWIR × A)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="33" t="inlineStr">
-        <is>
-          <t>I2</t>
-        </is>
-      </c>
-      <c r="B6" s="5" t="inlineStr">
-        <is>
-          <t>Fillings per year</t>
-        </is>
-      </c>
-      <c r="C6" s="25">
-        <f>IF(StageAreaVolume!B20=0,"",C5/StageAreaVolume!B20)</f>
-        <v/>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>I1 / crest storage</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="33" t="inlineStr">
-        <is>
-          <t>I3</t>
-        </is>
-      </c>
-      <c r="B7" s="5" t="inlineStr">
-        <is>
-          <t>Mean MDWIR</t>
-        </is>
-      </c>
-      <c r="C7" s="18">
-        <f>DailyCalc!S1</f>
-        <v/>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>mm/day</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
-        <is>
-          <t>Average dry-day infiltration rate</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="34" t="inlineStr"/>
-      <c r="B8" s="5" t="inlineStr">
-        <is>
-          <t>Mean E while ponded</t>
-        </is>
-      </c>
-      <c r="C8" s="18">
-        <f>IFERROR(AVERAGEIF(DailyCalc!C5:C204,"&gt;0",DailyCalc!G5:G204),0)</f>
-        <v/>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>mm/day</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
-        <is>
-          <t>Evaporation on days with water</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="34" t="inlineStr"/>
-      <c r="B9" s="5" t="inlineStr">
-        <is>
-          <t>MDWIR / E</t>
-        </is>
-      </c>
-      <c r="C9" s="25">
-        <f>IF(C8=0,"",C7/C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>Healthy gravel beds are often 4–8</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="33" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B10" s="5" t="inlineStr">
-        <is>
-          <t>Extra water-table rise vs control</t>
-        </is>
-      </c>
-      <c r="C10" s="25">
-        <f>Wells!L17</f>
-        <v/>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
-        <is>
-          <t>Mean Δh of W-N and W-M minus mean Δh of C</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="34" t="inlineStr"/>
-      <c r="B11" s="5" t="inlineStr">
-        <is>
-          <t>Recharge depth (Sy default)</t>
-        </is>
-      </c>
-      <c r="C11" s="18">
-        <f>Wells!L18</f>
-        <v/>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
-        <is>
-          <t>Sy × I4; not a volume</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
-      <c r="A12" s="34" t="inlineStr"/>
-      <c r="B12" s="5" t="inlineStr">
-        <is>
-          <t>Recharge depth range</t>
-        </is>
-      </c>
-      <c r="C12" s="35">
-        <f>TEXT(Wells!L19,"0.0")&amp;" – "&amp;TEXT(Wells!L20,"0.0")</f>
-        <v/>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>Sy low to Sy high</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="22" customHeight="1">
-      <c r="A13" s="33" t="inlineStr">
-        <is>
-          <t>I5</t>
-        </is>
-      </c>
-      <c r="B13" s="5" t="inlineStr">
-        <is>
-          <t>Extra karez flow-day visits</t>
-        </is>
-      </c>
-      <c r="C13" s="25">
-        <f>Karez!I7</f>
-        <v/>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>visits</t>
-        </is>
-      </c>
-      <c r="E13" s="6" t="inlineStr">
-        <is>
-          <t>Treated flowing visits − control flowing visits</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="22" customHeight="1">
-      <c r="A14" s="34" t="inlineStr"/>
-      <c r="B14" s="5" t="inlineStr">
-        <is>
-          <t>Extra karez days if weekly</t>
-        </is>
-      </c>
-      <c r="C14" s="25">
-        <f>C13*7</f>
-        <v/>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>days</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
-        <is>
-          <t>Assumes weekly KO visits</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="22" customHeight="1">
-      <c r="A15" s="34" t="inlineStr"/>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>Mean KO discharge while flowing</t>
-        </is>
-      </c>
-      <c r="C15" s="25">
-        <f>Karez!I5</f>
-        <v/>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>L/s</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
-        <is>
-          <t>Average of Q &gt; 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="22" customHeight="1">
-      <c r="A16" s="34" t="inlineStr"/>
-      <c r="B16" s="5" t="inlineStr">
-        <is>
-          <t>Days with water in pond</t>
-        </is>
-      </c>
-      <c r="C16" s="25">
-        <f>DailyCalc!S3</f>
-        <v/>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>days</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
-        <is>
-          <t>Stage &gt; 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="22" customHeight="1">
-      <c r="A17" s="34" t="inlineStr"/>
-      <c r="B17" s="5" t="inlineStr">
-        <is>
-          <t>Dry days used for MDWIR</t>
-        </is>
-      </c>
-      <c r="C17" s="25">
-        <f>DailyCalc!S4</f>
-        <v/>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>days</t>
-        </is>
-      </c>
-      <c r="E17" s="6" t="inlineStr">
-        <is>
-          <t>Should be as many as possible</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="22" customHeight="1">
-      <c r="A18" s="34" t="inlineStr"/>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>Crest storage</t>
-        </is>
-      </c>
-      <c r="C18" s="18">
+          <t>Rainfall to fill 100% and days water will stay</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="36" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Design hold is about 1–3 months when full. Yellow = assumptions. Blue uses Site catchment (ha) and crest V, A from StageAreaVolume. See docs/STORAGE_DURATION_AND_FILLING.md. SCS-CN: USDA-NRCS NEH-630.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3"/>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Inputs (yellow)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="inlineStr">
+        <is>
+          <t>Curve number CN</t>
+        </is>
+      </c>
+      <c r="B6" s="16" t="n">
+        <v>70</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>70–85 rocky rangeland; 60–75 fair pasture</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>Runoff coefficient C</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>First look only; 0.08–0.30 typical dryland</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="inlineStr">
+        <is>
+          <t>Initial abstraction ratio λ</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>0.20 standard SCS; try 0.05 in arid lands</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>Extra loss while filling (fraction)</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Infiltration + E during the fill storm</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>Volume already in pond (m³)</t>
+        </is>
+      </c>
+      <c r="B10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>0 if starting empty</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Open-water E (mm/day)</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Pan × 0.7; winter lower, summer higher</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="inlineStr">
+        <is>
+          <t>Bed infiltration i (mm/day)</t>
+        </is>
+      </c>
+      <c r="B12" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Use MDWIR once you have Form B</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>Wall/outlet leak (m³/day)</t>
+        </is>
+      </c>
+      <c r="B13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>0 if masonry and drain closed</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Results (blue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="inlineStr">
+        <is>
+          <t>Crest storage V (m³)</t>
+        </is>
+      </c>
+      <c r="B16" s="18">
         <f>StageAreaVolume!B20</f>
         <v/>
       </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
-        <is>
-          <t>From survey</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="22" customHeight="1">
-      <c r="A19" s="34" t="inlineStr"/>
-      <c r="B19" s="5" t="inlineStr">
-        <is>
-          <t>Catchment rain in DailyPond</t>
-        </is>
-      </c>
-      <c r="C19" s="18">
-        <f>SUM(DailyPond!B5:B204)</f>
-        <v/>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>Village gauge total for logged days</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="22" customHeight="1">
-      <c r="A20" s="34" t="inlineStr"/>
-      <c r="B20" s="5" t="inlineStr">
-        <is>
-          <t>I1 as depth on catchment</t>
-        </is>
-      </c>
-      <c r="C20" s="18">
-        <f>IF(Site!B14=0,"",C5/(Site!B14*10))</f>
-        <v/>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>mm</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>m³ / (ha × 10) = mm</t>
-        </is>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>Crest water area A (m²)</t>
+        </is>
+      </c>
+      <c r="B17" s="19">
+        <f>StageAreaVolume!B21</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="10" t="inlineStr">
+        <is>
+          <t>Catchment area (m²)</t>
+        </is>
+      </c>
+      <c r="B18" s="19">
+        <f>Site!B14*10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>Volume still needed (m³)</t>
+        </is>
+      </c>
+      <c r="B19" s="18">
+        <f>(B16-B10)*(1+B9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="10" t="inlineStr">
+        <is>
+          <t>Required runoff depth Q (mm)</t>
+        </is>
+      </c>
+      <c r="B20" s="25">
+        <f>IF(B18=0,"",B19/B18*1000)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>P to fill, constant C (mm)</t>
+        </is>
+      </c>
+      <c r="B21" s="18">
+        <f>IF(OR(B7=0,B20=""),"",B20/B7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>SCS S (mm)</t>
+        </is>
+      </c>
+      <c r="B22" s="18">
+        <f>IF(OR(B6&lt;=0,B6&gt;=100),"",25400/B6-254)</f>
+        <v/>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
-        <is>
-          <t>Workbook vs independent Python check (example dataset only)</t>
-        </is>
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>SCS Ia (mm)</t>
+        </is>
+      </c>
+      <c r="B23" s="18">
+        <f>IF(B22="","",B8*B22)</f>
+        <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>Python I1 (m³)</t>
-        </is>
-      </c>
-      <c r="B24" s="18" t="n">
-        <v>6365.418698335041</v>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>Workbook I1 − Python</t>
-        </is>
-      </c>
-      <c r="D24" s="18">
-        <f>C5-B24</f>
+      <c r="A24" s="10" t="inlineStr">
+        <is>
+          <t>P to fill, SCS-CN (mm)</t>
+        </is>
+      </c>
+      <c r="B24" s="18">
+        <f>IF(OR(B20="",B22=""),"",IF(B20&lt;=0,B23,B23+(B20+SQRT(B20^2+4*B20*B22))/2))</f>
         <v/>
       </c>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>Python mean MDWIR (mm/d)</t>
-        </is>
-      </c>
-      <c r="B25" s="25" t="n">
-        <v>48.21522767955886</v>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>Workbook MDWIR − Python</t>
-        </is>
-      </c>
-      <c r="D25" s="25">
-        <f>C7-B25</f>
+      <c r="A25" s="10" t="inlineStr">
+        <is>
+          <t>Capacity as mm on catchment</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>IF(B18=0,"",B16/B18*1000)</f>
         <v/>
       </c>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>Python I4 (m)</t>
-        </is>
-      </c>
-      <c r="B26" s="36" t="n">
-        <v>1.025</v>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Workbook I4 − Python</t>
-        </is>
-      </c>
-      <c r="D26" s="36">
-        <f>C10-B26</f>
+      <c r="A26" s="10" t="inlineStr">
+        <is>
+          <t>Days to empty, full area (shortest)</t>
+        </is>
+      </c>
+      <c r="B26" s="18">
+        <f>IF((B11+B12)/1000*B17+B13&lt;=0,"",B16/((B11+B12)/1000*B17+B13))</f>
         <v/>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>If the example is still loaded, differences should be near zero (interpolation rounding &lt; ~2%). After you replace the example, ignore this block.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>Days to empty, mean area (mid)</t>
+        </is>
+      </c>
+      <c r="B27" s="18">
+        <f>IF((B11+B12)/1000*(B17/2)+B13&lt;=0,"",B16/((B11+B12)/1000*(B17/2)+B13))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="12" t="inlineStr">
+        <is>
+          <t>P to fill is ONE storm from a dry catchment. Many 5–10 mm showers may never fill the dam if each is below Ia. Days to empty assume no further inflow and no pumping. Full-area days is a low estimate; mean-area is closer to a shrinking pond. Compare B26–B27 with the 30–90 day design. If B26 is &lt;&lt; 30, the bed is too leaky or the pond is too shallow. If I/E is near 1, you have an evaporation pan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31"/>
+    <row r="32"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A27:E28"/>
-    <mergeCell ref="A2:D2"/>
+  <mergeCells count="3">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E3"/>
+    <mergeCell ref="A29:E32"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="1" fitToWidth="1"/>

</xml_diff>